<commit_message>
mingle_users.xlsx Added new users
Added new users
</commit_message>
<xml_diff>
--- a/mingle_users.xlsx
+++ b/mingle_users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marialda/Library/Mobile Documents/com~apple~CloudDocs/Documents/Marialda/Resume/Everything else/GP/SD_RDO_6884/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2096BDDB-4806-B84E-BC57-77B36C6F2337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86AF5077-CFA8-7E4F-828B-11C066CC248B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="21440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5460" yWindow="1740" windowWidth="26640" windowHeight="19380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="46">
   <si>
     <t>First Name</t>
   </si>
@@ -52,12 +52,6 @@
     <t>Skill</t>
   </si>
   <si>
-    <t>marialda</t>
-  </si>
-  <si>
-    <t>cabral</t>
-  </si>
-  <si>
     <t>Coding</t>
   </si>
   <si>
@@ -73,9 +67,6 @@
     <t>doe</t>
   </si>
   <si>
-    <t>Coffee</t>
-  </si>
-  <si>
     <t>Bird Watching</t>
   </si>
   <si>
@@ -149,6 +140,24 @@
   </si>
   <si>
     <t>Tap Dancing</t>
+  </si>
+  <si>
+    <t>kay</t>
+  </si>
+  <si>
+    <t>moss</t>
+  </si>
+  <si>
+    <t>ella</t>
+  </si>
+  <si>
+    <t>wood</t>
+  </si>
+  <si>
+    <t>maria</t>
+  </si>
+  <si>
+    <t>fry</t>
   </si>
 </sst>
 </file>
@@ -512,11 +521,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="8" max="8" width="25.33203125" customWidth="1"/>
-    <col min="9" max="9" width="36.33203125" customWidth="1"/>
+    <col min="3" max="3" width="27.83203125" customWidth="1"/>
+    <col min="5" max="5" width="33.1640625" customWidth="1"/>
+    <col min="9" max="9" width="19.6640625" customWidth="1"/>
+    <col min="10" max="10" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -553,53 +564,50 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -607,13 +615,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -621,13 +629,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D6">
         <v>2</v>
@@ -635,36 +643,36 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -672,34 +680,56 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" t="s">
         <v>37</v>
       </c>
-      <c r="F9" t="s">
+      <c r="I9" t="s">
         <v>38</v>
       </c>
-      <c r="G9" t="s">
+      <c r="J9" t="s">
         <v>39</v>
       </c>
-      <c r="H9" t="s">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>40</v>
       </c>
-      <c r="I9" t="s">
+      <c r="B10" t="s">
         <v>41</v>
       </c>
-      <c r="J9" t="s">
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>